<commit_message>
Merge the two lookup tables into one Catalogue sheet
The output carried Sheet7 and Sheet9 because the reference workbook split
its ERP extract across two tabs, and the offer sheets VLOOKUP into them.
The names meant nothing to anyone who had not built that workbook, and an
upload with no ABS codes left Sheet9 empty in the delivered file.

Item codes are unique across the extract, so one table serves every offer
sheet. SheetSpec.source stays per-sheet, so a second table can still be
introduced from config.py if two suppliers ever collide on a code.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/template/pricing_tool_template.xlsx
+++ b/template/pricing_tool_template.xlsx
@@ -13,8 +13,7 @@
     <sheet name="O (UE3)" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="O (UE4)" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="Summary" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Sheet7" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Sheet9" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Catalogue" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'O (UE)'!$2:$2</definedName>
@@ -541,23 +540,6 @@
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table1" displayName="Table1" ref="A1:H2" headerRowCount="1" totalsRowShown="0">
   <autoFilter ref="A1:H73"/>
-  <tableColumns count="8">
-    <tableColumn id="18" name="Item No.1"/>
-    <tableColumn id="19" name="Description"/>
-    <tableColumn id="21" name="Unit Price"/>
-    <tableColumn id="24" name="Advanced Reserved"/>
-    <tableColumn id="26" name="Stock Available Quantity"/>
-    <tableColumn id="32" name="PO Qty"/>
-    <tableColumn id="33" name="PO not Shipped"/>
-    <tableColumn id="38" name="Landed USD"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</table>
-</file>
-
-<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Table13" displayName="Table13" ref="A1:H2" headerRowCount="1" totalsRowShown="0">
-  <autoFilter ref="A1:H18"/>
   <tableColumns count="8">
     <tableColumn id="18" name="Item No.1"/>
     <tableColumn id="19" name="Description"/>
@@ -3056,83 +3038,4 @@
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </tableParts>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:H2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="18.140625" bestFit="1" customWidth="1" min="1" max="1"/>
-    <col width="36.28515625" bestFit="1" customWidth="1" min="2" max="2"/>
-    <col width="11.28515625" bestFit="1" customWidth="1" min="3" max="3"/>
-    <col width="20" bestFit="1" customWidth="1" min="4" max="4"/>
-    <col width="24.140625" bestFit="1" customWidth="1" min="5" max="5"/>
-    <col width="9" bestFit="1" customWidth="1" min="6" max="6"/>
-    <col width="16.42578125" bestFit="1" customWidth="1" min="7" max="7"/>
-    <col width="13.42578125" bestFit="1" customWidth="1" min="8" max="8"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="64" t="inlineStr">
-        <is>
-          <t>Item No.1</t>
-        </is>
-      </c>
-      <c r="B1" s="64" t="inlineStr">
-        <is>
-          <t>Description</t>
-        </is>
-      </c>
-      <c r="C1" s="64" t="inlineStr">
-        <is>
-          <t>Unit Price</t>
-        </is>
-      </c>
-      <c r="D1" s="64" t="inlineStr">
-        <is>
-          <t>Advanced Reserved</t>
-        </is>
-      </c>
-      <c r="E1" s="64" t="inlineStr">
-        <is>
-          <t>Stock Available Quantity</t>
-        </is>
-      </c>
-      <c r="F1" s="64" t="inlineStr">
-        <is>
-          <t>PO Qty</t>
-        </is>
-      </c>
-      <c r="G1" s="64" t="inlineStr">
-        <is>
-          <t>PO not Shipped</t>
-        </is>
-      </c>
-      <c r="H1" s="64" t="inlineStr">
-        <is>
-          <t>Landed USD</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="65" t="n"/>
-      <c r="B2" s="65" t="n"/>
-      <c r="C2" s="9" t="n"/>
-      <c r="D2" s="9" t="n"/>
-      <c r="E2" s="9" t="n"/>
-      <c r="F2" s="9" t="n"/>
-      <c r="G2" s="9" t="n"/>
-      <c r="H2" s="9" t="n"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-  </tableParts>
-</worksheet>
 </file>
</xml_diff>